<commit_message>
Met a jour TP1-Portée-FoxTrot.xlsx
</commit_message>
<xml_diff>
--- a/TP1-Portée-FoxTrot.xlsx
+++ b/TP1-Portée-FoxTrot.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Utilisateur\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{173D84FD-8FB9-4E58-945B-0CC15999C2E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2E2F1459-4F4A-4763-B171-2F3116679E50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{3EEAE50F-06B8-FA41-A5DD-B39B708C16FA}"/>
   </bookViews>
@@ -42,7 +42,7 @@
     <author>tc={42065218-D621-D642-A3D3-09BE83CE3FAD}</author>
   </authors>
   <commentList>
-    <comment ref="A5" authorId="0" shapeId="0" xr:uid="{3574B8EC-C9E0-3647-9406-6CD5376AD160}">
+    <comment ref="A10" authorId="0" shapeId="0" xr:uid="{3574B8EC-C9E0-3647-9406-6CD5376AD160}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -50,7 +50,7 @@
     Inscrire le numéro de l'issue dans GitLab ou votre autre outil</t>
       </text>
     </comment>
-    <comment ref="F5" authorId="1" shapeId="0" xr:uid="{42065218-D621-D642-A3D3-09BE83CE3FAD}">
+    <comment ref="F10" authorId="1" shapeId="0" xr:uid="{42065218-D621-D642-A3D3-09BE83CE3FAD}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -63,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="56">
   <si>
     <t>INF6150-Été-2026</t>
   </si>
@@ -95,6 +95,9 @@
     <t>Pas commencé</t>
   </si>
   <si>
+    <t>Membre de l'equipe: Sileye Lamine Guisse - GUIS08369403</t>
+  </si>
+  <si>
     <t>Modification</t>
   </si>
   <si>
@@ -104,19 +107,49 @@
     <t>En raffinement</t>
   </si>
   <si>
+    <t>Mouhamed Rassoul Guiro - GUIM73340206</t>
+  </si>
+  <si>
+    <t>Aboubacar Niang - NIAA86340105</t>
+  </si>
+  <si>
+    <t>Bogue</t>
+  </si>
+  <si>
+    <t>Souhaitable</t>
+  </si>
+  <si>
+    <t>Prêt à développer</t>
+  </si>
+  <si>
+    <t>Ibrahima Berete - BERI75290402</t>
+  </si>
+  <si>
+    <t>Module</t>
+  </si>
+  <si>
+    <t>À déterminer</t>
+  </si>
+  <si>
+    <t>En développement</t>
+  </si>
+  <si>
+    <t>Marius Guimatsia Akalong -GUIM27309006</t>
+  </si>
+  <si>
+    <t>En vérification</t>
+  </si>
+  <si>
+    <t>En validation</t>
+  </si>
+  <si>
     <t>Liste des exigences de la portée initiale</t>
   </si>
   <si>
     <t xml:space="preserve">USP </t>
   </si>
   <si>
-    <t>Bogue</t>
-  </si>
-  <si>
-    <t>Souhaitable</t>
-  </si>
-  <si>
-    <t>Prêt à développer</t>
+    <t>Terminé</t>
   </si>
   <si>
     <t>#Exigence</t>
@@ -137,34 +170,16 @@
     <t>Notre contribution à date</t>
   </si>
   <si>
-    <t>Module</t>
-  </si>
-  <si>
-    <t>À déterminer</t>
-  </si>
-  <si>
-    <t>En développement</t>
-  </si>
-  <si>
     <t>Gérer les comptes utilisateurs</t>
   </si>
   <si>
     <t>Création et raffinement initial de l'exigence dans le cadre de l'élaboration du carnet de produit.</t>
   </si>
   <si>
-    <t>En vérification</t>
-  </si>
-  <si>
     <t>Gérer les véhicules</t>
   </si>
   <si>
-    <t>En validation</t>
-  </si>
-  <si>
     <t>Gérer les rendez-vous</t>
-  </si>
-  <si>
-    <t>Terminé</t>
   </si>
   <si>
     <t>Créer une demande de réparation</t>
@@ -253,7 +268,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -284,6 +299,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="10">
     <border>
@@ -406,7 +427,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -426,6 +447,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -646,8 +668,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{3022F5EC-73A9-E448-8905-B3FEE991BEF9}" name="Tableau3" displayName="Tableau3" ref="A5:G25" totalsRowShown="0" headerRowDxfId="10" headerRowBorderDxfId="8" tableBorderDxfId="9" totalsRowBorderDxfId="7">
-  <autoFilter ref="A5:G25" xr:uid="{3022F5EC-73A9-E448-8905-B3FEE991BEF9}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{3022F5EC-73A9-E448-8905-B3FEE991BEF9}" name="Tableau3" displayName="Tableau3" ref="A10:G30" totalsRowShown="0" headerRowDxfId="10" headerRowBorderDxfId="8" tableBorderDxfId="9" totalsRowBorderDxfId="7">
+  <autoFilter ref="A10:G30" xr:uid="{3022F5EC-73A9-E448-8905-B3FEE991BEF9}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{2E3D5560-96E8-064D-835F-7AF2DE0BAF44}" name="#Exigence" dataDxfId="6"/>
     <tableColumn id="2" xr3:uid="{8EF570CC-5B7D-8344-9CBB-A6FB8E1D38A1}" name="Titre résumé  de l'exigence" dataDxfId="5"/>
@@ -978,10 +1000,10 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="A5" dT="2026-01-21T19:06:43.28" personId="{3CBA3D62-BA07-F14D-8E55-850B9879B50E}" id="{3574B8EC-C9E0-3647-9406-6CD5376AD160}">
+  <threadedComment ref="A10" dT="2026-01-21T19:06:43.28" personId="{3CBA3D62-BA07-F14D-8E55-850B9879B50E}" id="{3574B8EC-C9E0-3647-9406-6CD5376AD160}">
     <text>Inscrire le numéro de l'issue dans GitLab ou votre autre outil</text>
   </threadedComment>
-  <threadedComment ref="F5" dT="2026-01-21T19:21:39.02" personId="{3CBA3D62-BA07-F14D-8E55-850B9879B50E}" id="{42065218-D621-D642-A3D3-09BE83CE3FAD}">
+  <threadedComment ref="F10" dT="2026-01-21T19:21:39.02" personId="{3CBA3D62-BA07-F14D-8E55-850B9879B50E}" id="{42065218-D621-D642-A3D3-09BE83CE3FAD}">
     <text>Indiquer au-dessus si c'est en USP (User Story Points) ou en PFC (Points de Fonction COSMIC).</text>
   </threadedComment>
 </ThreadedComments>
@@ -989,14 +1011,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0EC2CE87-59F9-6D4F-9E71-D5DBA81B5C36}">
-  <dimension ref="A1:N25"/>
+  <dimension ref="A1:N30"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6"/>
   <cols>
     <col min="1" max="1" width="9.75" customWidth="1"/>
     <col min="2" max="2" width="37.25" customWidth="1"/>
     <col min="3" max="3" width="16.25" customWidth="1"/>
     <col min="5" max="5" width="18.75" customWidth="1"/>
-    <col min="6" max="6" width="15.25" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.25" customWidth="1"/>
     <col min="7" max="7" width="75.375" customWidth="1"/>
     <col min="8" max="8" width="9.25" customWidth="1"/>
     <col min="11" max="11" width="15.75" bestFit="1" customWidth="1"/>
@@ -1005,15 +1027,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17" t="s">
+      <c r="B1" s="18"/>
+      <c r="C1" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
       <c r="K1" s="14" t="s">
         <v>2</v>
       </c>
@@ -1025,17 +1047,17 @@
       </c>
     </row>
     <row r="2" spans="1:14">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17" t="s">
+      <c r="B2" s="18"/>
+      <c r="C2" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
       <c r="K2" t="s">
         <v>7</v>
       </c>
@@ -1047,210 +1069,143 @@
       </c>
     </row>
     <row r="3" spans="1:14">
-      <c r="C3" s="1"/>
+      <c r="C3" s="1" t="s">
+        <v>10</v>
+      </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
       <c r="K3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="L3" s="8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="M3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" ht="21">
-      <c r="A4" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="B4" s="19"/>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="13" t="s">
+    </row>
+    <row r="4" spans="1:14">
+      <c r="C4" s="1"/>
+      <c r="D4" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="G4" s="13"/>
-      <c r="H4" s="13"/>
-      <c r="K4" t="s">
+      <c r="E4" s="1"/>
+      <c r="F4" s="1"/>
+      <c r="G4" s="1"/>
+      <c r="L4" s="8"/>
+    </row>
+    <row r="5" spans="1:14" ht="15.75">
+      <c r="C5" s="1"/>
+      <c r="D5" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="L4" s="9" t="s">
+      <c r="E5" s="1"/>
+      <c r="F5" s="1"/>
+      <c r="G5" s="1"/>
+      <c r="K5" t="s">
         <v>16</v>
       </c>
-      <c r="M4" t="s">
+      <c r="L5" s="9" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="5" spans="1:14">
-      <c r="A5" s="15" t="s">
+      <c r="M5" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="12" t="s">
+    </row>
+    <row r="6" spans="1:14" ht="15.75">
+      <c r="C6" s="1"/>
+      <c r="D6" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C5" s="12" t="s">
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
+      <c r="K6" t="s">
         <v>20</v>
       </c>
-      <c r="D5" s="12" t="s">
+      <c r="L6" t="s">
         <v>21</v>
       </c>
-      <c r="E5" s="16" t="s">
+      <c r="M6" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" ht="15.75">
+      <c r="C7" s="1"/>
+      <c r="D7" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E7" s="1"/>
+      <c r="F7" s="1"/>
+      <c r="G7" s="1"/>
+      <c r="L7" s="17"/>
+      <c r="M7" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" ht="15.75">
+      <c r="C8" s="1"/>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
+      <c r="F8" s="1"/>
+      <c r="G8" s="1"/>
+      <c r="L8" s="17"/>
+      <c r="M8" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" ht="21">
+      <c r="A9" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="B9" s="20"/>
+      <c r="C9" s="20"/>
+      <c r="D9" s="20"/>
+      <c r="E9" s="20"/>
+      <c r="F9" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="G9" s="13"/>
+      <c r="H9" s="13"/>
+      <c r="M9" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14">
+      <c r="A10" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="B10" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C10" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="D10" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="E10" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="F5" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="G5" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="K5" t="s">
-        <v>24</v>
-      </c>
-      <c r="L5" t="s">
-        <v>25</v>
-      </c>
-      <c r="M5" t="s">
-        <v>26</v>
-      </c>
-      <c r="N5" s="10"/>
-    </row>
-    <row r="6" spans="1:14">
-      <c r="A6" s="3">
-        <v>1</v>
-      </c>
-      <c r="B6" t="s">
-        <v>27</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="F6" s="11">
-        <v>8</v>
-      </c>
-      <c r="G6" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="M6" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14">
-      <c r="A7" s="3">
-        <v>2</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="F7" s="2">
-        <v>5</v>
-      </c>
-      <c r="G7" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="M7" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14">
-      <c r="A8" s="3">
-        <v>3</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="F8" s="2">
-        <v>13</v>
-      </c>
-      <c r="G8" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="M8" t="s">
+      <c r="F10" s="12" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="9" spans="1:14">
-      <c r="A9" s="3">
-        <v>4</v>
-      </c>
-      <c r="B9" s="2" t="s">
+      <c r="G10" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="C9" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="F9" s="2">
-        <v>8</v>
-      </c>
-      <c r="G9" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="M9" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14">
-      <c r="A10" s="3">
-        <v>5</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="F10" s="2">
-        <v>8</v>
-      </c>
-      <c r="G10" s="11" t="s">
-        <v>28</v>
-      </c>
+      <c r="M10" t="s">
+        <v>21</v>
+      </c>
+      <c r="N10" s="10"/>
     </row>
     <row r="11" spans="1:14">
       <c r="A11" s="3">
-        <v>6</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>36</v>
+        <v>1</v>
+      </c>
+      <c r="B11" t="s">
+        <v>35</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>7</v>
@@ -1261,22 +1216,22 @@
       <c r="E11" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="F11" s="2">
-        <v>13</v>
+      <c r="F11" s="11">
+        <v>8</v>
       </c>
       <c r="G11" s="11" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
     </row>
     <row r="12" spans="1:14">
       <c r="A12" s="3">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>37</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>8</v>
@@ -1285,15 +1240,15 @@
         <v>9</v>
       </c>
       <c r="F12" s="2">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="G12" s="11" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
     </row>
     <row r="13" spans="1:14">
       <c r="A13" s="3">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>38</v>
@@ -1302,21 +1257,21 @@
         <v>7</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E13" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F13" s="2">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="G13" s="11" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
     </row>
     <row r="14" spans="1:14">
       <c r="A14" s="3">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>39</v>
@@ -1325,7 +1280,7 @@
         <v>7</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E14" s="4" t="s">
         <v>9</v>
@@ -1334,12 +1289,12 @@
         <v>8</v>
       </c>
       <c r="G14" s="11" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
     </row>
     <row r="15" spans="1:14">
       <c r="A15" s="3">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>40</v>
@@ -1348,7 +1303,7 @@
         <v>7</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E15" s="4" t="s">
         <v>9</v>
@@ -1357,12 +1312,12 @@
         <v>8</v>
       </c>
       <c r="G15" s="11" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
     </row>
     <row r="16" spans="1:14">
       <c r="A16" s="3">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>41</v>
@@ -1371,243 +1326,358 @@
         <v>7</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E16" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F16" s="2">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="G16" s="11" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
     </row>
     <row r="17" spans="1:7">
       <c r="A17" s="3">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>42</v>
       </c>
       <c r="C17" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F17" s="2">
+        <v>13</v>
+      </c>
+      <c r="G17" s="11" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7">
+      <c r="A18" s="3">
+        <v>8</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C18" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D17" s="2" t="s">
+      <c r="D18" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F18" s="2">
+        <v>8</v>
+      </c>
+      <c r="G18" s="11" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7">
+      <c r="A19" s="3">
+        <v>9</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F19" s="2">
+        <v>8</v>
+      </c>
+      <c r="G19" s="11" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7">
+      <c r="A20" s="3">
+        <v>10</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F20" s="2">
+        <v>8</v>
+      </c>
+      <c r="G20" s="11" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7">
+      <c r="A21" s="3">
         <v>11</v>
       </c>
-      <c r="E17" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="F17" s="2">
-        <v>8</v>
-      </c>
-      <c r="G17" s="11" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7">
-      <c r="A18" s="5">
-        <v>13</v>
-      </c>
-      <c r="B18" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="C18" s="6" t="s">
+      <c r="B21" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C21" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D18" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="E18" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="F18" s="6">
+      <c r="D21" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F21" s="2">
         <v>5</v>
       </c>
-      <c r="G18" s="11" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7">
-      <c r="A19" s="5">
-        <v>14</v>
-      </c>
-      <c r="B19" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="C19" s="6" t="s">
+      <c r="G21" s="11" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7">
+      <c r="A22" s="3">
+        <v>12</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C22" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D19" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="E19" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="F19" s="6">
-        <v>5</v>
-      </c>
-      <c r="G19" s="11" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7">
-      <c r="A20" s="5">
-        <v>15</v>
-      </c>
-      <c r="B20" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="C20" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="D20" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="E20" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="F20" s="6">
-        <v>13</v>
-      </c>
-      <c r="G20" s="11" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7">
-      <c r="A21" s="5">
-        <v>16</v>
-      </c>
-      <c r="B21" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="C21" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="D21" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E21" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="F21" s="6">
-        <v>8</v>
-      </c>
-      <c r="G21" s="11" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7">
-      <c r="A22" s="5">
-        <v>17</v>
-      </c>
-      <c r="B22" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="C22" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="D22" s="6" t="s">
-        <v>16</v>
+      <c r="D22" s="2" t="s">
+        <v>12</v>
       </c>
       <c r="E22" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="F22" s="6">
-        <v>5</v>
+      <c r="F22" s="2">
+        <v>8</v>
       </c>
       <c r="G22" s="11" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
     </row>
     <row r="23" spans="1:7">
       <c r="A23" s="5">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="B23" s="6" t="s">
         <v>48</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="E23" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F23" s="6">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="G23" s="11" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
     </row>
     <row r="24" spans="1:7">
       <c r="A24" s="5">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="B24" s="6" t="s">
         <v>49</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="E24" s="4" t="s">
         <v>9</v>
       </c>
       <c r="F24" s="6">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="G24" s="11" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
     </row>
     <row r="25" spans="1:7">
       <c r="A25" s="5">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="B25" s="6" t="s">
         <v>50</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D25" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E25" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F25" s="6">
+        <v>13</v>
+      </c>
+      <c r="G25" s="11" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7">
+      <c r="A26" s="5">
         <v>16</v>
       </c>
-      <c r="E25" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="F25" s="6">
-        <v>8</v>
-      </c>
-      <c r="G25" s="11" t="s">
-        <v>28</v>
+      <c r="B26" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F26" s="6">
+        <v>8</v>
+      </c>
+      <c r="G26" s="11" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7">
+      <c r="A27" s="5">
+        <v>17</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="D27" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="E27" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F27" s="6">
+        <v>5</v>
+      </c>
+      <c r="G27" s="11" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7">
+      <c r="A28" s="5">
+        <v>18</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="D28" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F28" s="6">
+        <v>13</v>
+      </c>
+      <c r="G28" s="11" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7">
+      <c r="A29" s="5">
+        <v>19</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="D29" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="E29" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F29" s="6">
+        <v>13</v>
+      </c>
+      <c r="G29" s="11" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7">
+      <c r="A30" s="5">
+        <v>20</v>
+      </c>
+      <c r="B30" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="C30" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="D30" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="E30" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F30" s="6">
+        <v>8</v>
+      </c>
+      <c r="G30" s="11" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="C1:E1"/>
     <mergeCell ref="C2:G2"/>
-    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="A9:E9"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A2:B2"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C6:C25" xr:uid="{D4651FD4-E6DB-9748-9F7C-DE0F67AABCCB}">
-      <formula1>$K$2:$K$5</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C11:C30" xr:uid="{D4651FD4-E6DB-9748-9F7C-DE0F67AABCCB}">
+      <formula1>$K$2:$K$9</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D6:D25" xr:uid="{381BE1F6-DFC4-E543-8C05-33687E42ABA5}">
-      <formula1>$L$2:$L$5</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D11:D30" xr:uid="{381BE1F6-DFC4-E543-8C05-33687E42ABA5}">
+      <formula1>$L$2:$L$9</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E6:E25" xr:uid="{73079421-D23E-4045-92D6-531B890FF9E1}">
-      <formula1>$M$2:$M$9</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E11:E30" xr:uid="{73079421-D23E-4045-92D6-531B890FF9E1}">
+      <formula1>$M$2:$M$13</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>